<commit_message>
Add cards-grid block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 13
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-reagents.report.xlsx
+++ b/tools/importer/reports/import-reagents.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="53">
   <si>
     <t>_reportFile</t>
   </si>
@@ -79,7 +79,7 @@
     <t>reagents/centrifugation</t>
   </si>
   <si>
-    <t>2026-10-27T07:47:48.322Z</t>
+    <t>2026-10-27T10:14:30.018Z</t>
   </si>
   <si>
     <t>Centrifugation</t>
@@ -131,6 +131,45 @@
   </si>
   <si>
     <t>https://www.mybeckman.in/reagents/particle</t>
+  </si>
+  <si>
+    <t>reagents/particle/valita-aggregation-pure.report.json</t>
+  </si>
+  <si>
+    <t>["content-product-detail","columns-features","embed-video","cards-grid","cards-resource-list","cards-doc-table"]</t>
+  </si>
+  <si>
+    <t>reagents/particle/valita-aggregation-pure</t>
+  </si>
+  <si>
+    <t>reagent-product</t>
+  </si>
+  <si>
+    <t>2026-10-27T08:31:50.377Z</t>
+  </si>
+  <si>
+    <t>Valita Aggregation Pure Assays to determine Protein Aggregation</t>
+  </si>
+  <si>
+    <t>https://www.mybeckman.in/reagents/particle/valita-aggregation-pure</t>
+  </si>
+  <si>
+    <t>reagents/particle/valita-titer-assays.report.json</t>
+  </si>
+  <si>
+    <t>["content-product-detail","columns-features","hero","embed-video","columns-icon-list","cards-grid","content-reversed","cards-resource-list","cards-doc-table"]</t>
+  </si>
+  <si>
+    <t>reagents/particle/valita-titer-assays</t>
+  </si>
+  <si>
+    <t>2026-10-27T08:31:47.747Z</t>
+  </si>
+  <si>
+    <t>Valita Titer Assays for IgG Quantification</t>
+  </si>
+  <si>
+    <t>https://www.mybeckman.in/reagents/particle/valita-titer-assays</t>
   </si>
 </sst>
 </file>
@@ -519,13 +558,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="43" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
@@ -712,6 +750,58 @@
         <v>39</v>
       </c>
     </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>